<commit_message>
Data wrangling - allele data cleaning
Ran HWE-MAF QC on filtered data as well - all OK, although p values are smaller after filtering for baseline overweight.
</commit_message>
<xml_diff>
--- a/dataprep/experiment_allele_integration_24Jun26/Pronokal_DatosGenomics_Desencriptado_1Jul26.xlsx
+++ b/dataprep/experiment_allele_integration_24Jun26/Pronokal_DatosGenomics_Desencriptado_1Jul26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imdea-my.sharepoint.com/personal/miksa_henkrich_nutricion_imdea_org/Documents/Escritorio/PNK/dataprep/experiment_allele_integration_24Jun26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{A4F03186-1E6F-43FB-AC29-E4D5CAF2F91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{286EC277-D66D-4C3B-AA74-6BC9966726ED}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{A4F03186-1E6F-43FB-AC29-E4D5CAF2F91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{391DFBDC-99F7-4CD8-B8E6-AE7A32698FB9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{4C3DB20B-D0C1-44F0-81F5-4740EE862306}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12628" uniqueCount="12628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12624" uniqueCount="12624">
   <si>
     <t>ID Paciente</t>
   </si>
@@ -37911,18 +37911,6 @@
   </si>
   <si>
     <t>CG Desencriptado</t>
-  </si>
-  <si>
-    <t>post march rows in old</t>
-  </si>
-  <si>
-    <t>post march rows in new</t>
-  </si>
-  <si>
-    <t>row diff</t>
-  </si>
-  <si>
-    <t>sample diff</t>
   </si>
 </sst>
 </file>
@@ -38317,7 +38305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45179A13-23E2-4335-BBBD-59959953CAAE}">
-  <dimension ref="A1:H4208"/>
+  <dimension ref="A1:C4208"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="46.88671875" customWidth="1"/>
@@ -84259,7 +84247,7 @@
         <v>8440</v>
       </c>
     </row>
-    <row r="4177" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4177" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4177" t="s">
         <v>3619</v>
       </c>
@@ -84270,7 +84258,7 @@
         <v>10224</v>
       </c>
     </row>
-    <row r="4178" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4178" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4178" t="s">
         <v>3303</v>
       </c>
@@ -84281,7 +84269,7 @@
         <v>10066</v>
       </c>
     </row>
-    <row r="4179" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4179" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4179" t="s">
         <v>3607</v>
       </c>
@@ -84292,7 +84280,7 @@
         <v>10218</v>
       </c>
     </row>
-    <row r="4180" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4180" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4180" t="s">
         <v>3437</v>
       </c>
@@ -84303,7 +84291,7 @@
         <v>10133</v>
       </c>
     </row>
-    <row r="4181" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4181" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4181" t="s">
         <v>2739</v>
       </c>
@@ -84314,7 +84302,7 @@
         <v>9784</v>
       </c>
     </row>
-    <row r="4182" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4182" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4182" t="s">
         <v>652</v>
       </c>
@@ -84325,7 +84313,7 @@
         <v>8742</v>
       </c>
     </row>
-    <row r="4183" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4183" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4183" t="s">
         <v>16</v>
       </c>
@@ -84336,7 +84324,7 @@
         <v>8424</v>
       </c>
     </row>
-    <row r="4184" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4184" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4184" t="s">
         <v>1698</v>
       </c>
@@ -84347,7 +84335,7 @@
         <v>9265</v>
       </c>
     </row>
-    <row r="4185" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4185" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4185" t="s">
         <v>2475</v>
       </c>
@@ -84358,7 +84346,7 @@
         <v>9652</v>
       </c>
     </row>
-    <row r="4186" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4186" t="s">
         <v>3339</v>
       </c>
@@ -84369,7 +84357,7 @@
         <v>10084</v>
       </c>
     </row>
-    <row r="4187" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4187" t="s">
         <v>3633</v>
       </c>
@@ -84380,7 +84368,7 @@
         <v>10231</v>
       </c>
     </row>
-    <row r="4188" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4188" t="s">
         <v>3319</v>
       </c>
@@ -84390,15 +84378,8 @@
       <c r="C4188" t="s">
         <v>10074</v>
       </c>
-      <c r="F4188" t="s">
-        <v>12624</v>
-      </c>
-      <c r="H4188">
-        <f>72759-23343</f>
-        <v>49416</v>
-      </c>
-    </row>
-    <row r="4189" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4189" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4189" t="s">
         <v>3421</v>
       </c>
@@ -84408,15 +84389,8 @@
       <c r="C4189" t="s">
         <v>10125</v>
       </c>
-      <c r="F4189" t="s">
-        <v>12625</v>
-      </c>
-      <c r="H4189">
-        <f>57840-13340</f>
-        <v>44500</v>
-      </c>
-    </row>
-    <row r="4190" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4190" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4190" t="s">
         <v>3601</v>
       </c>
@@ -84426,15 +84400,8 @@
       <c r="C4190" t="s">
         <v>10215</v>
       </c>
-      <c r="F4190" t="s">
-        <v>12626</v>
-      </c>
-      <c r="H4190">
-        <f>H4188-H4189</f>
-        <v>4916</v>
-      </c>
-    </row>
-    <row r="4191" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4191" t="s">
         <v>3641</v>
       </c>
@@ -84444,15 +84411,8 @@
       <c r="C4191" t="s">
         <v>10235</v>
       </c>
-      <c r="F4191" t="s">
-        <v>12627</v>
-      </c>
-      <c r="H4191">
-        <f>H4190/20</f>
-        <v>245.8</v>
-      </c>
-    </row>
-    <row r="4192" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4192" t="s">
         <v>3389</v>
       </c>
@@ -84463,7 +84423,7 @@
         <v>10109</v>
       </c>
     </row>
-    <row r="4193" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4193" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4193" t="s">
         <v>46</v>
       </c>
@@ -84473,12 +84433,8 @@
       <c r="C4193" t="s">
         <v>8439</v>
       </c>
-      <c r="F4193">
-        <f>46040/20</f>
-        <v>2302</v>
-      </c>
-    </row>
-    <row r="4194" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4194" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4194" t="s">
         <v>906</v>
       </c>
@@ -84489,7 +84445,7 @@
         <v>8869</v>
       </c>
     </row>
-    <row r="4195" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4195" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4195" t="s">
         <v>1832</v>
       </c>
@@ -84500,7 +84456,7 @@
         <v>9331</v>
       </c>
     </row>
-    <row r="4196" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4196" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4196" t="s">
         <v>660</v>
       </c>
@@ -84511,7 +84467,7 @@
         <v>8746</v>
       </c>
     </row>
-    <row r="4197" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4197" t="s">
         <v>3461</v>
       </c>
@@ -84522,7 +84478,7 @@
         <v>10145</v>
       </c>
     </row>
-    <row r="4198" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4198" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4198" t="s">
         <v>668</v>
       </c>
@@ -84533,7 +84489,7 @@
         <v>8750</v>
       </c>
     </row>
-    <row r="4199" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4199" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4199" t="s">
         <v>3213</v>
       </c>
@@ -84544,7 +84500,7 @@
         <v>10021</v>
       </c>
     </row>
-    <row r="4200" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4200" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4200" t="s">
         <v>2645</v>
       </c>
@@ -84555,7 +84511,7 @@
         <v>9737</v>
       </c>
     </row>
-    <row r="4201" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4201" t="s">
         <v>3609</v>
       </c>
@@ -84566,7 +84522,7 @@
         <v>10219</v>
       </c>
     </row>
-    <row r="4202" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4202" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4202" t="s">
         <v>1110</v>
       </c>
@@ -84577,7 +84533,7 @@
         <v>8971</v>
       </c>
     </row>
-    <row r="4203" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4203" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4203" t="s">
         <v>3321</v>
       </c>
@@ -84588,7 +84544,7 @@
         <v>10075</v>
       </c>
     </row>
-    <row r="4204" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4204" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4204" t="s">
         <v>3441</v>
       </c>
@@ -84599,7 +84555,7 @@
         <v>10135</v>
       </c>
     </row>
-    <row r="4205" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4205" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4205" t="s">
         <v>2917</v>
       </c>
@@ -84610,7 +84566,7 @@
         <v>9873</v>
       </c>
     </row>
-    <row r="4206" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4206" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4206" t="s">
         <v>3495</v>
       </c>
@@ -84621,7 +84577,7 @@
         <v>10162</v>
       </c>
     </row>
-    <row r="4207" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4207" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4207" t="s">
         <v>3175</v>
       </c>
@@ -84632,7 +84588,7 @@
         <v>10002</v>
       </c>
     </row>
-    <row r="4208" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4208" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4208" t="s">
         <v>1770</v>
       </c>

</xml_diff>